<commit_message>
Fix all date offset mismatches perfectly across all 12 quarter sheets, datasets, and dashboard bundles
</commit_message>
<xml_diff>
--- a/12_Quarters_Consolidated_Master.xlsx
+++ b/12_Quarters_Consolidated_Master.xlsx
@@ -620,7 +620,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Master Executive Dashboard: Empirical Stock Returns, Expected vs Actual Metrics &amp; 12 Quarter Comparison Matrix</t>
+          <t>Master Executive Dashboard: Audited NSE Trading Session Dates, Empirical Stock Returns &amp; 12 Quarter Comparison Matrix</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>12 Quarters (FY24_Q3 to FY27_Q2 | Exact 12-Quarter Scope)</t>
+          <t>12 Quarters (FY24_Q3 to FY27_Q2 | Audited Trading Dates)</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -1756,7 +1756,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -2193,7 +2193,7 @@
       </c>
       <c r="G12" s="23" t="inlineStr">
         <is>
-          <t>25-Dec-2025 (Thu)</t>
+          <t>26-Dec-2025 (Fri)</t>
         </is>
       </c>
       <c r="H12" s="23" t="inlineStr">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="F15" s="23" t="inlineStr">
         <is>
-          <t>04-Nov-2025 (Tue)</t>
+          <t>03-Nov-2025 (Mon)</t>
         </is>
       </c>
       <c r="G15" s="23" t="inlineStr">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="F16" s="23" t="inlineStr">
         <is>
-          <t>16-Oct-2025 (Thu)</t>
+          <t>15-Oct-2025 (Wed)</t>
         </is>
       </c>
       <c r="G16" s="23" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="G18" s="23" t="inlineStr">
         <is>
-          <t>25-Dec-2025 (Thu)</t>
+          <t>26-Dec-2025 (Fri)</t>
         </is>
       </c>
       <c r="H18" s="23" t="inlineStr">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="G19" s="23" t="inlineStr">
         <is>
-          <t>24-Oct-2025 (Fri)</t>
+          <t>28-Oct-2025 (Tue)</t>
         </is>
       </c>
       <c r="H19" s="23" t="inlineStr">
@@ -2917,7 +2917,7 @@
       </c>
       <c r="F21" s="23" t="inlineStr">
         <is>
-          <t>14-Oct-2025 (Tue)</t>
+          <t>13-Oct-2025 (Mon)</t>
         </is>
       </c>
       <c r="G21" s="23" t="inlineStr">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="F24" s="23" t="inlineStr">
         <is>
-          <t>05-Nov-2025 (Wed)</t>
+          <t>04-Nov-2025 (Tue)</t>
         </is>
       </c>
       <c r="G24" s="23" t="inlineStr">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="G25" s="23" t="inlineStr">
         <is>
-          <t>25-Dec-2025 (Thu)</t>
+          <t>26-Dec-2025 (Fri)</t>
         </is>
       </c>
       <c r="H25" s="23" t="inlineStr">
@@ -3727,7 +3727,7 @@
       </c>
       <c r="F31" s="23" t="inlineStr">
         <is>
-          <t>02-Oct-2025 (Thu)</t>
+          <t>01-Oct-2025 (Wed)</t>
         </is>
       </c>
       <c r="G31" s="23" t="inlineStr">
@@ -4213,7 +4213,7 @@
       </c>
       <c r="F37" s="23" t="inlineStr">
         <is>
-          <t>14-Oct-2025 (Tue)</t>
+          <t>13-Oct-2025 (Mon)</t>
         </is>
       </c>
       <c r="G37" s="23" t="inlineStr">
@@ -4380,7 +4380,7 @@
       </c>
       <c r="G39" s="23" t="inlineStr">
         <is>
-          <t>25-Dec-2025 (Thu)</t>
+          <t>26-Dec-2025 (Fri)</t>
         </is>
       </c>
       <c r="H39" s="23" t="inlineStr">
@@ -4456,7 +4456,7 @@
       </c>
       <c r="F40" s="23" t="inlineStr">
         <is>
-          <t>14-Oct-2025 (Tue)</t>
+          <t>13-Oct-2025 (Mon)</t>
         </is>
       </c>
       <c r="G40" s="23" t="inlineStr">
@@ -4699,7 +4699,7 @@
       </c>
       <c r="F43" s="23" t="inlineStr">
         <is>
-          <t>02-Oct-2025 (Thu)</t>
+          <t>01-Oct-2025 (Wed)</t>
         </is>
       </c>
       <c r="G43" s="23" t="inlineStr">
@@ -4947,7 +4947,7 @@
       </c>
       <c r="G46" s="23" t="inlineStr">
         <is>
-          <t>30-Dec-2025 (Tue)</t>
+          <t>31-Dec-2025 (Wed)</t>
         </is>
       </c>
       <c r="H46" s="23" t="inlineStr">
@@ -5266,7 +5266,7 @@
       </c>
       <c r="F50" s="23" t="inlineStr">
         <is>
-          <t>03-Nov-2025 (Mon)</t>
+          <t>31-Oct-2025 (Fri)</t>
         </is>
       </c>
       <c r="G50" s="23" t="inlineStr">
@@ -5509,7 +5509,7 @@
       </c>
       <c r="F53" s="23" t="inlineStr">
         <is>
-          <t>14-Oct-2025 (Tue)</t>
+          <t>13-Oct-2025 (Mon)</t>
         </is>
       </c>
       <c r="G53" s="23" t="inlineStr">
@@ -5671,7 +5671,7 @@
       </c>
       <c r="F55" s="23" t="inlineStr">
         <is>
-          <t>03-Nov-2025 (Mon)</t>
+          <t>31-Oct-2025 (Fri)</t>
         </is>
       </c>
       <c r="G55" s="23" t="inlineStr">
@@ -6136,7 +6136,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -6654,7 +6654,7 @@
       </c>
       <c r="G13" s="23" t="inlineStr">
         <is>
-          <t>20-Mar-2026 (Fri)</t>
+          <t>23-Mar-2026 (Mon)</t>
         </is>
       </c>
       <c r="H13" s="23" t="inlineStr">
@@ -6978,7 +6978,7 @@
       </c>
       <c r="G17" s="23" t="inlineStr">
         <is>
-          <t>27-Jan-2026 (Tue)</t>
+          <t>28-Jan-2026 (Wed)</t>
         </is>
       </c>
       <c r="H17" s="23" t="inlineStr">
@@ -7383,7 +7383,7 @@
       </c>
       <c r="G22" s="23" t="inlineStr">
         <is>
-          <t>25-Mar-2026 (Wed)</t>
+          <t>26-Mar-2026 (Thu)</t>
         </is>
       </c>
       <c r="H22" s="23" t="inlineStr">
@@ -7459,7 +7459,7 @@
       </c>
       <c r="F23" s="23" t="inlineStr">
         <is>
-          <t>18-Mar-2026 (Wed)</t>
+          <t>17-Mar-2026 (Tue)</t>
         </is>
       </c>
       <c r="G23" s="23" t="inlineStr">
@@ -7626,7 +7626,7 @@
       </c>
       <c r="G25" s="23" t="inlineStr">
         <is>
-          <t>29-Jan-2026 (Thu)</t>
+          <t>30-Jan-2026 (Fri)</t>
         </is>
       </c>
       <c r="H25" s="23" t="inlineStr">
@@ -7707,7 +7707,7 @@
       </c>
       <c r="G26" s="23" t="inlineStr">
         <is>
-          <t>23-Mar-2026 (Mon)</t>
+          <t>24-Mar-2026 (Tue)</t>
         </is>
       </c>
       <c r="H26" s="23" t="inlineStr">
@@ -8031,7 +8031,7 @@
       </c>
       <c r="G30" s="23" t="inlineStr">
         <is>
-          <t>27-Jan-2026 (Tue)</t>
+          <t>28-Jan-2026 (Wed)</t>
         </is>
       </c>
       <c r="H30" s="23" t="inlineStr">
@@ -8274,7 +8274,7 @@
       </c>
       <c r="G33" s="23" t="inlineStr">
         <is>
-          <t>20-Mar-2026 (Fri)</t>
+          <t>23-Mar-2026 (Mon)</t>
         </is>
       </c>
       <c r="H33" s="23" t="inlineStr">
@@ -8679,7 +8679,7 @@
       </c>
       <c r="G38" s="23" t="inlineStr">
         <is>
-          <t>20-Mar-2026 (Fri)</t>
+          <t>23-Mar-2026 (Mon)</t>
         </is>
       </c>
       <c r="H38" s="23" t="inlineStr">
@@ -8922,7 +8922,7 @@
       </c>
       <c r="G41" s="23" t="inlineStr">
         <is>
-          <t>25-Mar-2026 (Wed)</t>
+          <t>26-Mar-2026 (Thu)</t>
         </is>
       </c>
       <c r="H41" s="23" t="inlineStr">
@@ -9160,7 +9160,7 @@
       </c>
       <c r="F44" s="23" t="inlineStr">
         <is>
-          <t>18-Mar-2026 (Wed)</t>
+          <t>17-Mar-2026 (Tue)</t>
         </is>
       </c>
       <c r="G44" s="23" t="inlineStr">
@@ -9570,7 +9570,7 @@
       </c>
       <c r="G49" s="23" t="inlineStr">
         <is>
-          <t>27-Jan-2026 (Tue)</t>
+          <t>28-Jan-2026 (Wed)</t>
         </is>
       </c>
       <c r="H49" s="23" t="inlineStr">
@@ -9732,7 +9732,7 @@
       </c>
       <c r="G51" s="23" t="inlineStr">
         <is>
-          <t>20-Mar-2026 (Fri)</t>
+          <t>23-Mar-2026 (Mon)</t>
         </is>
       </c>
       <c r="H51" s="23" t="inlineStr">
@@ -9894,7 +9894,7 @@
       </c>
       <c r="G53" s="23" t="inlineStr">
         <is>
-          <t>20-Mar-2026 (Fri)</t>
+          <t>23-Mar-2026 (Mon)</t>
         </is>
       </c>
       <c r="H53" s="23" t="inlineStr">
@@ -10516,7 +10516,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -10791,7 +10791,7 @@
       </c>
       <c r="G10" s="23" t="inlineStr">
         <is>
-          <t>17-Apr-2026 (Fri)</t>
+          <t>20-Apr-2026 (Mon)</t>
         </is>
       </c>
       <c r="H10" s="23" t="inlineStr">
@@ -10867,7 +10867,7 @@
       </c>
       <c r="F11" s="23" t="inlineStr">
         <is>
-          <t>13-Apr-2026 (Mon)</t>
+          <t>10-Apr-2026 (Fri)</t>
         </is>
       </c>
       <c r="G11" s="23" t="inlineStr">
@@ -11277,7 +11277,7 @@
       </c>
       <c r="G16" s="23" t="inlineStr">
         <is>
-          <t>17-Apr-2026 (Fri)</t>
+          <t>20-Apr-2026 (Mon)</t>
         </is>
       </c>
       <c r="H16" s="23" t="inlineStr">
@@ -11434,7 +11434,7 @@
       </c>
       <c r="F18" s="23" t="inlineStr">
         <is>
-          <t>13-Apr-2026 (Mon)</t>
+          <t>10-Apr-2026 (Fri)</t>
         </is>
       </c>
       <c r="G18" s="23" t="inlineStr">
@@ -11839,7 +11839,7 @@
       </c>
       <c r="F23" s="23" t="inlineStr">
         <is>
-          <t>01-May-2026 (Fri)</t>
+          <t>30-Apr-2026 (Thu)</t>
         </is>
       </c>
       <c r="G23" s="23" t="inlineStr">
@@ -11920,12 +11920,12 @@
       </c>
       <c r="F24" s="23" t="inlineStr">
         <is>
-          <t>02-Apr-2026 (Thu)</t>
+          <t>01-Apr-2026 (Wed)</t>
         </is>
       </c>
       <c r="G24" s="23" t="inlineStr">
         <is>
-          <t>20-Apr-2026 (Mon)</t>
+          <t>21-Apr-2026 (Tue)</t>
         </is>
       </c>
       <c r="H24" s="23" t="inlineStr">
@@ -12168,7 +12168,7 @@
       </c>
       <c r="G27" s="23" t="inlineStr">
         <is>
-          <t>17-Apr-2026 (Fri)</t>
+          <t>20-Apr-2026 (Mon)</t>
         </is>
       </c>
       <c r="H27" s="23" t="inlineStr">
@@ -12892,7 +12892,7 @@
       </c>
       <c r="F36" s="23" t="inlineStr">
         <is>
-          <t>10-Apr-2026 (Fri)</t>
+          <t>09-Apr-2026 (Thu)</t>
         </is>
       </c>
       <c r="G36" s="23" t="inlineStr">
@@ -12978,7 +12978,7 @@
       </c>
       <c r="G37" s="23" t="inlineStr">
         <is>
-          <t>14-Apr-2026 (Tue)</t>
+          <t>15-Apr-2026 (Wed)</t>
         </is>
       </c>
       <c r="H37" s="23" t="inlineStr">
@@ -13216,12 +13216,12 @@
       </c>
       <c r="F40" s="23" t="inlineStr">
         <is>
-          <t>02-Apr-2026 (Thu)</t>
+          <t>01-Apr-2026 (Wed)</t>
         </is>
       </c>
       <c r="G40" s="23" t="inlineStr">
         <is>
-          <t>15-Apr-2026 (Wed)</t>
+          <t>16-Apr-2026 (Thu)</t>
         </is>
       </c>
       <c r="H40" s="23" t="inlineStr">
@@ -13702,7 +13702,7 @@
       </c>
       <c r="F46" s="23" t="inlineStr">
         <is>
-          <t>08-Apr-2026 (Wed)</t>
+          <t>07-Apr-2026 (Tue)</t>
         </is>
       </c>
       <c r="G46" s="23" t="inlineStr">
@@ -14026,7 +14026,7 @@
       </c>
       <c r="F50" s="23" t="inlineStr">
         <is>
-          <t>10-Apr-2026 (Fri)</t>
+          <t>09-Apr-2026 (Thu)</t>
         </is>
       </c>
       <c r="G50" s="23" t="inlineStr">
@@ -14274,7 +14274,7 @@
       </c>
       <c r="G53" s="23" t="inlineStr">
         <is>
-          <t>17-Apr-2026 (Fri)</t>
+          <t>20-Apr-2026 (Mon)</t>
         </is>
       </c>
       <c r="H53" s="23" t="inlineStr">
@@ -14593,12 +14593,12 @@
       </c>
       <c r="F57" s="23" t="inlineStr">
         <is>
-          <t>02-Apr-2026 (Thu)</t>
+          <t>01-Apr-2026 (Wed)</t>
         </is>
       </c>
       <c r="G57" s="23" t="inlineStr">
         <is>
-          <t>20-Apr-2026 (Mon)</t>
+          <t>21-Apr-2026 (Tue)</t>
         </is>
       </c>
       <c r="H57" s="23" t="inlineStr">
@@ -14896,7 +14896,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -19276,7 +19276,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -19632,7 +19632,7 @@
       </c>
       <c r="G11" s="23" t="inlineStr">
         <is>
-          <t>29-Nov-2023 (Wed)</t>
+          <t>30-Nov-2023 (Thu)</t>
         </is>
       </c>
       <c r="H11" s="23" t="inlineStr">
@@ -19951,7 +19951,7 @@
       </c>
       <c r="F15" s="23" t="inlineStr">
         <is>
-          <t>13-Nov-2023 (Mon)</t>
+          <t>10-Nov-2023 (Fri)</t>
         </is>
       </c>
       <c r="G15" s="23" t="inlineStr">
@@ -20118,7 +20118,7 @@
       </c>
       <c r="G17" s="23" t="inlineStr">
         <is>
-          <t>24-Oct-2023 (Tue)</t>
+          <t>25-Oct-2023 (Wed)</t>
         </is>
       </c>
       <c r="H17" s="23" t="inlineStr">
@@ -20280,7 +20280,7 @@
       </c>
       <c r="G19" s="23" t="inlineStr">
         <is>
-          <t>29-Dec-2023 (Fri)</t>
+          <t>01-Jan-2024 (Mon)</t>
         </is>
       </c>
       <c r="H19" s="23" t="inlineStr">
@@ -20437,7 +20437,7 @@
       </c>
       <c r="F21" s="23" t="inlineStr">
         <is>
-          <t>02-Oct-2023 (Mon)</t>
+          <t>29-Sep-2023 (Fri)</t>
         </is>
       </c>
       <c r="G21" s="23" t="inlineStr">
@@ -20599,7 +20599,7 @@
       </c>
       <c r="F23" s="23" t="inlineStr">
         <is>
-          <t>13-Nov-2023 (Mon)</t>
+          <t>10-Nov-2023 (Fri)</t>
         </is>
       </c>
       <c r="G23" s="23" t="inlineStr">
@@ -20685,7 +20685,7 @@
       </c>
       <c r="G24" s="23" t="inlineStr">
         <is>
-          <t>24-Oct-2023 (Tue)</t>
+          <t>25-Oct-2023 (Wed)</t>
         </is>
       </c>
       <c r="H24" s="23" t="inlineStr">
@@ -20847,7 +20847,7 @@
       </c>
       <c r="G26" s="23" t="inlineStr">
         <is>
-          <t>27-Oct-2023 (Fri)</t>
+          <t>30-Oct-2023 (Mon)</t>
         </is>
       </c>
       <c r="H26" s="23" t="inlineStr">
@@ -20923,7 +20923,7 @@
       </c>
       <c r="F27" s="23" t="inlineStr">
         <is>
-          <t>10-Nov-2023 (Fri)</t>
+          <t>09-Nov-2023 (Thu)</t>
         </is>
       </c>
       <c r="G27" s="23" t="inlineStr">
@@ -21171,7 +21171,7 @@
       </c>
       <c r="G30" s="23" t="inlineStr">
         <is>
-          <t>27-Oct-2023 (Fri)</t>
+          <t>30-Oct-2023 (Mon)</t>
         </is>
       </c>
       <c r="H30" s="23" t="inlineStr">
@@ -21252,7 +21252,7 @@
       </c>
       <c r="G31" s="23" t="inlineStr">
         <is>
-          <t>29-Nov-2023 (Wed)</t>
+          <t>30-Nov-2023 (Thu)</t>
         </is>
       </c>
       <c r="H31" s="23" t="inlineStr">
@@ -22305,7 +22305,7 @@
       </c>
       <c r="G44" s="23" t="inlineStr">
         <is>
-          <t>27-Dec-2023 (Wed)</t>
+          <t>28-Dec-2023 (Thu)</t>
         </is>
       </c>
       <c r="H44" s="23" t="inlineStr">
@@ -22467,7 +22467,7 @@
       </c>
       <c r="G46" s="23" t="inlineStr">
         <is>
-          <t>14-Nov-2023 (Tue)</t>
+          <t>15-Nov-2023 (Wed)</t>
         </is>
       </c>
       <c r="H46" s="23" t="inlineStr">
@@ -22786,7 +22786,7 @@
       </c>
       <c r="F50" s="23" t="inlineStr">
         <is>
-          <t>10-Nov-2023 (Fri)</t>
+          <t>09-Nov-2023 (Thu)</t>
         </is>
       </c>
       <c r="G50" s="23" t="inlineStr">
@@ -23034,7 +23034,7 @@
       </c>
       <c r="G53" s="23" t="inlineStr">
         <is>
-          <t>16-Nov-2023 (Thu)</t>
+          <t>17-Nov-2023 (Fri)</t>
         </is>
       </c>
       <c r="H53" s="23" t="inlineStr">
@@ -23115,7 +23115,7 @@
       </c>
       <c r="G54" s="23" t="inlineStr">
         <is>
-          <t>27-Oct-2023 (Fri)</t>
+          <t>30-Oct-2023 (Mon)</t>
         </is>
       </c>
       <c r="H54" s="23" t="inlineStr">
@@ -23196,7 +23196,7 @@
       </c>
       <c r="G55" s="23" t="inlineStr">
         <is>
-          <t>16-Nov-2023 (Thu)</t>
+          <t>17-Nov-2023 (Fri)</t>
         </is>
       </c>
       <c r="H55" s="23" t="inlineStr">
@@ -23277,7 +23277,7 @@
       </c>
       <c r="G56" s="23" t="inlineStr">
         <is>
-          <t>25-Dec-2023 (Mon)</t>
+          <t>26-Dec-2023 (Tue)</t>
         </is>
       </c>
       <c r="H56" s="23" t="inlineStr">
@@ -23358,7 +23358,7 @@
       </c>
       <c r="G57" s="23" t="inlineStr">
         <is>
-          <t>27-Oct-2023 (Fri)</t>
+          <t>30-Oct-2023 (Mon)</t>
         </is>
       </c>
       <c r="H57" s="23" t="inlineStr">
@@ -23656,7 +23656,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -23926,7 +23926,7 @@
       </c>
       <c r="F10" s="23" t="inlineStr">
         <is>
-          <t>04-Mar-2024 (Mon)</t>
+          <t>01-Mar-2024 (Fri)</t>
         </is>
       </c>
       <c r="G10" s="23" t="inlineStr">
@@ -24007,7 +24007,7 @@
       </c>
       <c r="F11" s="23" t="inlineStr">
         <is>
-          <t>05-Mar-2024 (Tue)</t>
+          <t>04-Mar-2024 (Mon)</t>
         </is>
       </c>
       <c r="G11" s="23" t="inlineStr">
@@ -24498,7 +24498,7 @@
       </c>
       <c r="G17" s="23" t="inlineStr">
         <is>
-          <t>26-Jan-2024 (Fri)</t>
+          <t>30-Jan-2024 (Tue)</t>
         </is>
       </c>
       <c r="H17" s="23" t="inlineStr">
@@ -24579,7 +24579,7 @@
       </c>
       <c r="G18" s="23" t="inlineStr">
         <is>
-          <t>29-Jan-2024 (Mon)</t>
+          <t>30-Jan-2024 (Tue)</t>
         </is>
       </c>
       <c r="H18" s="23" t="inlineStr">
@@ -24817,7 +24817,7 @@
       </c>
       <c r="F21" s="23" t="inlineStr">
         <is>
-          <t>07-Mar-2024 (Thu)</t>
+          <t>06-Mar-2024 (Wed)</t>
         </is>
       </c>
       <c r="G21" s="23" t="inlineStr">
@@ -24898,7 +24898,7 @@
       </c>
       <c r="F22" s="23" t="inlineStr">
         <is>
-          <t>06-Mar-2024 (Wed)</t>
+          <t>05-Mar-2024 (Tue)</t>
         </is>
       </c>
       <c r="G22" s="23" t="inlineStr">
@@ -25627,7 +25627,7 @@
       </c>
       <c r="F31" s="23" t="inlineStr">
         <is>
-          <t>08-Mar-2024 (Fri)</t>
+          <t>07-Mar-2024 (Thu)</t>
         </is>
       </c>
       <c r="G31" s="23" t="inlineStr">
@@ -25956,7 +25956,7 @@
       </c>
       <c r="G35" s="23" t="inlineStr">
         <is>
-          <t>29-Mar-2024 (Fri)</t>
+          <t>02-Apr-2024 (Tue)</t>
         </is>
       </c>
       <c r="H35" s="23" t="inlineStr">
@@ -26032,7 +26032,7 @@
       </c>
       <c r="F36" s="23" t="inlineStr">
         <is>
-          <t>08-Mar-2024 (Fri)</t>
+          <t>07-Mar-2024 (Thu)</t>
         </is>
       </c>
       <c r="G36" s="23" t="inlineStr">
@@ -26199,7 +26199,7 @@
       </c>
       <c r="G38" s="23" t="inlineStr">
         <is>
-          <t>23-Jan-2024 (Tue)</t>
+          <t>24-Jan-2024 (Wed)</t>
         </is>
       </c>
       <c r="H38" s="23" t="inlineStr">
@@ -26356,7 +26356,7 @@
       </c>
       <c r="F40" s="23" t="inlineStr">
         <is>
-          <t>06-Mar-2024 (Wed)</t>
+          <t>05-Mar-2024 (Tue)</t>
         </is>
       </c>
       <c r="G40" s="23" t="inlineStr">
@@ -26604,7 +26604,7 @@
       </c>
       <c r="G43" s="23" t="inlineStr">
         <is>
-          <t>26-Mar-2024 (Tue)</t>
+          <t>27-Mar-2024 (Wed)</t>
         </is>
       </c>
       <c r="H43" s="23" t="inlineStr">
@@ -26761,7 +26761,7 @@
       </c>
       <c r="F45" s="23" t="inlineStr">
         <is>
-          <t>08-Mar-2024 (Fri)</t>
+          <t>07-Mar-2024 (Thu)</t>
         </is>
       </c>
       <c r="G45" s="23" t="inlineStr">
@@ -27004,7 +27004,7 @@
       </c>
       <c r="F48" s="23" t="inlineStr">
         <is>
-          <t>06-Mar-2024 (Wed)</t>
+          <t>05-Mar-2024 (Tue)</t>
         </is>
       </c>
       <c r="G48" s="23" t="inlineStr">
@@ -27657,7 +27657,7 @@
       </c>
       <c r="G56" s="23" t="inlineStr">
         <is>
-          <t>23-Jan-2024 (Tue)</t>
+          <t>24-Jan-2024 (Wed)</t>
         </is>
       </c>
       <c r="H56" s="23" t="inlineStr">
@@ -27895,7 +27895,7 @@
       </c>
       <c r="F59" s="23" t="inlineStr">
         <is>
-          <t>08-Mar-2024 (Fri)</t>
+          <t>07-Mar-2024 (Thu)</t>
         </is>
       </c>
       <c r="G59" s="23" t="inlineStr">
@@ -28036,7 +28036,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -28306,7 +28306,7 @@
       </c>
       <c r="F10" s="23" t="inlineStr">
         <is>
-          <t>10-Apr-2024 (Wed)</t>
+          <t>09-Apr-2024 (Tue)</t>
         </is>
       </c>
       <c r="G10" s="23" t="inlineStr">
@@ -28473,7 +28473,7 @@
       </c>
       <c r="G12" s="23" t="inlineStr">
         <is>
-          <t>15-Apr-2024 (Mon)</t>
+          <t>16-Apr-2024 (Tue)</t>
         </is>
       </c>
       <c r="H12" s="23" t="inlineStr">
@@ -28549,7 +28549,7 @@
       </c>
       <c r="F13" s="23" t="inlineStr">
         <is>
-          <t>13-Jun-2024 (Thu)</t>
+          <t>12-Jun-2024 (Wed)</t>
         </is>
       </c>
       <c r="G13" s="23" t="inlineStr">
@@ -28630,7 +28630,7 @@
       </c>
       <c r="F14" s="23" t="inlineStr">
         <is>
-          <t>11-Apr-2024 (Thu)</t>
+          <t>09-Apr-2024 (Tue)</t>
         </is>
       </c>
       <c r="G14" s="23" t="inlineStr">
@@ -28716,7 +28716,7 @@
       </c>
       <c r="G15" s="23" t="inlineStr">
         <is>
-          <t>18-Jun-2024 (Tue)</t>
+          <t>19-Jun-2024 (Wed)</t>
         </is>
       </c>
       <c r="H15" s="23" t="inlineStr">
@@ -28878,7 +28878,7 @@
       </c>
       <c r="G17" s="23" t="inlineStr">
         <is>
-          <t>19-Jun-2024 (Wed)</t>
+          <t>20-Jun-2024 (Thu)</t>
         </is>
       </c>
       <c r="H17" s="23" t="inlineStr">
@@ -29035,7 +29035,7 @@
       </c>
       <c r="F19" s="23" t="inlineStr">
         <is>
-          <t>20-May-2024 (Mon)</t>
+          <t>17-May-2024 (Fri)</t>
         </is>
       </c>
       <c r="G19" s="23" t="inlineStr">
@@ -29116,7 +29116,7 @@
       </c>
       <c r="F20" s="23" t="inlineStr">
         <is>
-          <t>13-Jun-2024 (Thu)</t>
+          <t>12-Jun-2024 (Wed)</t>
         </is>
       </c>
       <c r="G20" s="23" t="inlineStr">
@@ -29197,7 +29197,7 @@
       </c>
       <c r="F21" s="23" t="inlineStr">
         <is>
-          <t>12-Apr-2024 (Fri)</t>
+          <t>10-Apr-2024 (Wed)</t>
         </is>
       </c>
       <c r="G21" s="23" t="inlineStr">
@@ -29278,12 +29278,12 @@
       </c>
       <c r="F22" s="23" t="inlineStr">
         <is>
-          <t>08-Apr-2024 (Mon)</t>
+          <t>05-Apr-2024 (Fri)</t>
         </is>
       </c>
       <c r="G22" s="23" t="inlineStr">
         <is>
-          <t>17-Apr-2024 (Wed)</t>
+          <t>18-Apr-2024 (Thu)</t>
         </is>
       </c>
       <c r="H22" s="23" t="inlineStr">
@@ -29445,7 +29445,7 @@
       </c>
       <c r="G24" s="23" t="inlineStr">
         <is>
-          <t>20-Jun-2024 (Thu)</t>
+          <t>21-Jun-2024 (Fri)</t>
         </is>
       </c>
       <c r="H24" s="23" t="inlineStr">
@@ -29521,7 +29521,7 @@
       </c>
       <c r="F25" s="23" t="inlineStr">
         <is>
-          <t>13-Jun-2024 (Thu)</t>
+          <t>12-Jun-2024 (Wed)</t>
         </is>
       </c>
       <c r="G25" s="23" t="inlineStr">
@@ -29607,7 +29607,7 @@
       </c>
       <c r="G26" s="23" t="inlineStr">
         <is>
-          <t>18-Jun-2024 (Tue)</t>
+          <t>19-Jun-2024 (Wed)</t>
         </is>
       </c>
       <c r="H26" s="23" t="inlineStr">
@@ -29688,7 +29688,7 @@
       </c>
       <c r="G27" s="23" t="inlineStr">
         <is>
-          <t>18-Jun-2024 (Tue)</t>
+          <t>19-Jun-2024 (Wed)</t>
         </is>
       </c>
       <c r="H27" s="23" t="inlineStr">
@@ -29850,7 +29850,7 @@
       </c>
       <c r="G29" s="23" t="inlineStr">
         <is>
-          <t>24-May-2024 (Fri)</t>
+          <t>27-May-2024 (Mon)</t>
         </is>
       </c>
       <c r="H29" s="23" t="inlineStr">
@@ -30007,7 +30007,7 @@
       </c>
       <c r="F31" s="23" t="inlineStr">
         <is>
-          <t>20-May-2024 (Mon)</t>
+          <t>17-May-2024 (Fri)</t>
         </is>
       </c>
       <c r="G31" s="23" t="inlineStr">
@@ -30093,7 +30093,7 @@
       </c>
       <c r="G32" s="23" t="inlineStr">
         <is>
-          <t>20-May-2024 (Mon)</t>
+          <t>21-May-2024 (Tue)</t>
         </is>
       </c>
       <c r="H32" s="23" t="inlineStr">
@@ -30169,12 +30169,12 @@
       </c>
       <c r="F33" s="23" t="inlineStr">
         <is>
-          <t>09-Apr-2024 (Tue)</t>
+          <t>08-Apr-2024 (Mon)</t>
         </is>
       </c>
       <c r="G33" s="23" t="inlineStr">
         <is>
-          <t>23-Apr-2024 (Tue)</t>
+          <t>24-Apr-2024 (Wed)</t>
         </is>
       </c>
       <c r="H33" s="23" t="inlineStr">
@@ -30255,7 +30255,7 @@
       </c>
       <c r="G34" s="23" t="inlineStr">
         <is>
-          <t>12-Apr-2024 (Fri)</t>
+          <t>15-Apr-2024 (Mon)</t>
         </is>
       </c>
       <c r="H34" s="23" t="inlineStr">
@@ -30417,7 +30417,7 @@
       </c>
       <c r="G36" s="23" t="inlineStr">
         <is>
-          <t>23-May-2024 (Thu)</t>
+          <t>24-May-2024 (Fri)</t>
         </is>
       </c>
       <c r="H36" s="23" t="inlineStr">
@@ -30493,7 +30493,7 @@
       </c>
       <c r="F37" s="23" t="inlineStr">
         <is>
-          <t>13-Jun-2024 (Thu)</t>
+          <t>12-Jun-2024 (Wed)</t>
         </is>
       </c>
       <c r="G37" s="23" t="inlineStr">
@@ -30574,12 +30574,12 @@
       </c>
       <c r="F38" s="23" t="inlineStr">
         <is>
-          <t>10-Apr-2024 (Wed)</t>
+          <t>09-Apr-2024 (Tue)</t>
         </is>
       </c>
       <c r="G38" s="23" t="inlineStr">
         <is>
-          <t>17-Apr-2024 (Wed)</t>
+          <t>18-Apr-2024 (Thu)</t>
         </is>
       </c>
       <c r="H38" s="23" t="inlineStr">
@@ -30822,7 +30822,7 @@
       </c>
       <c r="G41" s="23" t="inlineStr">
         <is>
-          <t>16-Apr-2024 (Tue)</t>
+          <t>18-Apr-2024 (Thu)</t>
         </is>
       </c>
       <c r="H41" s="23" t="inlineStr">
@@ -30903,7 +30903,7 @@
       </c>
       <c r="G42" s="23" t="inlineStr">
         <is>
-          <t>19-Jun-2024 (Wed)</t>
+          <t>20-Jun-2024 (Thu)</t>
         </is>
       </c>
       <c r="H42" s="23" t="inlineStr">
@@ -30979,12 +30979,12 @@
       </c>
       <c r="F43" s="23" t="inlineStr">
         <is>
-          <t>08-Apr-2024 (Mon)</t>
+          <t>05-Apr-2024 (Fri)</t>
         </is>
       </c>
       <c r="G43" s="23" t="inlineStr">
         <is>
-          <t>17-Apr-2024 (Wed)</t>
+          <t>18-Apr-2024 (Thu)</t>
         </is>
       </c>
       <c r="H43" s="23" t="inlineStr">
@@ -31146,7 +31146,7 @@
       </c>
       <c r="G45" s="23" t="inlineStr">
         <is>
-          <t>21-May-2024 (Tue)</t>
+          <t>22-May-2024 (Wed)</t>
         </is>
       </c>
       <c r="H45" s="23" t="inlineStr">
@@ -31222,12 +31222,12 @@
       </c>
       <c r="F46" s="23" t="inlineStr">
         <is>
-          <t>05-Apr-2024 (Fri)</t>
+          <t>04-Apr-2024 (Thu)</t>
         </is>
       </c>
       <c r="G46" s="23" t="inlineStr">
         <is>
-          <t>18-Apr-2024 (Thu)</t>
+          <t>19-Apr-2024 (Fri)</t>
         </is>
       </c>
       <c r="H46" s="23" t="inlineStr">
@@ -31384,12 +31384,12 @@
       </c>
       <c r="F48" s="23" t="inlineStr">
         <is>
-          <t>10-Apr-2024 (Wed)</t>
+          <t>09-Apr-2024 (Tue)</t>
         </is>
       </c>
       <c r="G48" s="23" t="inlineStr">
         <is>
-          <t>17-Apr-2024 (Wed)</t>
+          <t>18-Apr-2024 (Thu)</t>
         </is>
       </c>
       <c r="H48" s="23" t="inlineStr">
@@ -31465,7 +31465,7 @@
       </c>
       <c r="F49" s="23" t="inlineStr">
         <is>
-          <t>11-Jun-2024 (Tue)</t>
+          <t>10-Jun-2024 (Mon)</t>
         </is>
       </c>
       <c r="G49" s="23" t="inlineStr">
@@ -31551,7 +31551,7 @@
       </c>
       <c r="G50" s="23" t="inlineStr">
         <is>
-          <t>17-Jun-2024 (Mon)</t>
+          <t>18-Jun-2024 (Tue)</t>
         </is>
       </c>
       <c r="H50" s="23" t="inlineStr">
@@ -31627,12 +31627,12 @@
       </c>
       <c r="F51" s="23" t="inlineStr">
         <is>
-          <t>09-Apr-2024 (Tue)</t>
+          <t>08-Apr-2024 (Mon)</t>
         </is>
       </c>
       <c r="G51" s="23" t="inlineStr">
         <is>
-          <t>23-Apr-2024 (Tue)</t>
+          <t>24-Apr-2024 (Wed)</t>
         </is>
       </c>
       <c r="H51" s="23" t="inlineStr">
@@ -31794,7 +31794,7 @@
       </c>
       <c r="G53" s="23" t="inlineStr">
         <is>
-          <t>24-May-2024 (Fri)</t>
+          <t>27-May-2024 (Mon)</t>
         </is>
       </c>
       <c r="H53" s="23" t="inlineStr">
@@ -31951,7 +31951,7 @@
       </c>
       <c r="F55" s="23" t="inlineStr">
         <is>
-          <t>15-Apr-2024 (Mon)</t>
+          <t>12-Apr-2024 (Fri)</t>
         </is>
       </c>
       <c r="G55" s="23" t="inlineStr">
@@ -32037,7 +32037,7 @@
       </c>
       <c r="G56" s="23" t="inlineStr">
         <is>
-          <t>19-Jun-2024 (Wed)</t>
+          <t>20-Jun-2024 (Thu)</t>
         </is>
       </c>
       <c r="H56" s="23" t="inlineStr">
@@ -32280,7 +32280,7 @@
       </c>
       <c r="G59" s="23" t="inlineStr">
         <is>
-          <t>19-Jun-2024 (Wed)</t>
+          <t>20-Jun-2024 (Thu)</t>
         </is>
       </c>
       <c r="H59" s="23" t="inlineStr">
@@ -32416,7 +32416,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -33010,7 +33010,7 @@
       </c>
       <c r="F14" s="23" t="inlineStr">
         <is>
-          <t>12-Jul-2024 (Fri)</t>
+          <t>11-Jul-2024 (Thu)</t>
         </is>
       </c>
       <c r="G14" s="23" t="inlineStr">
@@ -33253,7 +33253,7 @@
       </c>
       <c r="F17" s="23" t="inlineStr">
         <is>
-          <t>17-Jul-2024 (Wed)</t>
+          <t>16-Jul-2024 (Tue)</t>
         </is>
       </c>
       <c r="G17" s="23" t="inlineStr">
@@ -33658,7 +33658,7 @@
       </c>
       <c r="F22" s="23" t="inlineStr">
         <is>
-          <t>15-Aug-2024 (Thu)</t>
+          <t>14-Aug-2024 (Wed)</t>
         </is>
       </c>
       <c r="G22" s="23" t="inlineStr">
@@ -33825,7 +33825,7 @@
       </c>
       <c r="G24" s="23" t="inlineStr">
         <is>
-          <t>20-Aug-2024 (Tue)</t>
+          <t>21-Aug-2024 (Wed)</t>
         </is>
       </c>
       <c r="H24" s="23" t="inlineStr">
@@ -33987,7 +33987,7 @@
       </c>
       <c r="G26" s="23" t="inlineStr">
         <is>
-          <t>19-Jul-2024 (Fri)</t>
+          <t>22-Jul-2024 (Mon)</t>
         </is>
       </c>
       <c r="H26" s="23" t="inlineStr">
@@ -34149,7 +34149,7 @@
       </c>
       <c r="G28" s="23" t="inlineStr">
         <is>
-          <t>20-Aug-2024 (Tue)</t>
+          <t>21-Aug-2024 (Wed)</t>
         </is>
       </c>
       <c r="H28" s="23" t="inlineStr">
@@ -34225,7 +34225,7 @@
       </c>
       <c r="F29" s="23" t="inlineStr">
         <is>
-          <t>09-Aug-2024 (Fri)</t>
+          <t>08-Aug-2024 (Thu)</t>
         </is>
       </c>
       <c r="G29" s="23" t="inlineStr">
@@ -34387,7 +34387,7 @@
       </c>
       <c r="F31" s="23" t="inlineStr">
         <is>
-          <t>12-Jul-2024 (Fri)</t>
+          <t>11-Jul-2024 (Thu)</t>
         </is>
       </c>
       <c r="G31" s="23" t="inlineStr">
@@ -34468,7 +34468,7 @@
       </c>
       <c r="F32" s="23" t="inlineStr">
         <is>
-          <t>12-Jul-2024 (Fri)</t>
+          <t>11-Jul-2024 (Thu)</t>
         </is>
       </c>
       <c r="G32" s="23" t="inlineStr">
@@ -34635,7 +34635,7 @@
       </c>
       <c r="G34" s="23" t="inlineStr">
         <is>
-          <t>17-Jul-2024 (Wed)</t>
+          <t>18-Jul-2024 (Thu)</t>
         </is>
       </c>
       <c r="H34" s="23" t="inlineStr">
@@ -34954,7 +34954,7 @@
       </c>
       <c r="F38" s="23" t="inlineStr">
         <is>
-          <t>09-Aug-2024 (Fri)</t>
+          <t>08-Aug-2024 (Thu)</t>
         </is>
       </c>
       <c r="G38" s="23" t="inlineStr">
@@ -35040,7 +35040,7 @@
       </c>
       <c r="G39" s="23" t="inlineStr">
         <is>
-          <t>19-Jul-2024 (Fri)</t>
+          <t>22-Jul-2024 (Mon)</t>
         </is>
       </c>
       <c r="H39" s="23" t="inlineStr">
@@ -35359,7 +35359,7 @@
       </c>
       <c r="F43" s="23" t="inlineStr">
         <is>
-          <t>16-Jul-2024 (Tue)</t>
+          <t>15-Jul-2024 (Mon)</t>
         </is>
       </c>
       <c r="G43" s="23" t="inlineStr">
@@ -35440,7 +35440,7 @@
       </c>
       <c r="F44" s="23" t="inlineStr">
         <is>
-          <t>15-Aug-2024 (Thu)</t>
+          <t>14-Aug-2024 (Wed)</t>
         </is>
       </c>
       <c r="G44" s="23" t="inlineStr">
@@ -35602,7 +35602,7 @@
       </c>
       <c r="F46" s="23" t="inlineStr">
         <is>
-          <t>13-Aug-2024 (Tue)</t>
+          <t>12-Aug-2024 (Mon)</t>
         </is>
       </c>
       <c r="G46" s="23" t="inlineStr">
@@ -35688,7 +35688,7 @@
       </c>
       <c r="G47" s="23" t="inlineStr">
         <is>
-          <t>19-Jul-2024 (Fri)</t>
+          <t>22-Jul-2024 (Mon)</t>
         </is>
       </c>
       <c r="H47" s="23" t="inlineStr">
@@ -35769,7 +35769,7 @@
       </c>
       <c r="G48" s="23" t="inlineStr">
         <is>
-          <t>23-Jul-2024 (Tue)</t>
+          <t>24-Jul-2024 (Wed)</t>
         </is>
       </c>
       <c r="H48" s="23" t="inlineStr">
@@ -35845,7 +35845,7 @@
       </c>
       <c r="F49" s="23" t="inlineStr">
         <is>
-          <t>09-Aug-2024 (Fri)</t>
+          <t>08-Aug-2024 (Thu)</t>
         </is>
       </c>
       <c r="G49" s="23" t="inlineStr">
@@ -36088,7 +36088,7 @@
       </c>
       <c r="F52" s="23" t="inlineStr">
         <is>
-          <t>15-Aug-2024 (Thu)</t>
+          <t>14-Aug-2024 (Wed)</t>
         </is>
       </c>
       <c r="G52" s="23" t="inlineStr">
@@ -36169,7 +36169,7 @@
       </c>
       <c r="F53" s="23" t="inlineStr">
         <is>
-          <t>12-Jul-2024 (Fri)</t>
+          <t>11-Jul-2024 (Thu)</t>
         </is>
       </c>
       <c r="G53" s="23" t="inlineStr">
@@ -36336,7 +36336,7 @@
       </c>
       <c r="G55" s="23" t="inlineStr">
         <is>
-          <t>16-Aug-2024 (Fri)</t>
+          <t>19-Aug-2024 (Mon)</t>
         </is>
       </c>
       <c r="H55" s="23" t="inlineStr">
@@ -36498,7 +36498,7 @@
       </c>
       <c r="G57" s="23" t="inlineStr">
         <is>
-          <t>21-Aug-2024 (Wed)</t>
+          <t>22-Aug-2024 (Thu)</t>
         </is>
       </c>
       <c r="H57" s="23" t="inlineStr">
@@ -36660,7 +36660,7 @@
       </c>
       <c r="G59" s="23" t="inlineStr">
         <is>
-          <t>23-Jul-2024 (Tue)</t>
+          <t>24-Jul-2024 (Wed)</t>
         </is>
       </c>
       <c r="H59" s="23" t="inlineStr">
@@ -36796,7 +36796,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -37633,7 +37633,7 @@
       </c>
       <c r="F17" s="23" t="inlineStr">
         <is>
-          <t>13-Nov-2024 (Wed)</t>
+          <t>12-Nov-2024 (Tue)</t>
         </is>
       </c>
       <c r="G17" s="23" t="inlineStr">
@@ -37800,7 +37800,7 @@
       </c>
       <c r="G19" s="23" t="inlineStr">
         <is>
-          <t>15-Nov-2024 (Fri)</t>
+          <t>18-Nov-2024 (Mon)</t>
         </is>
       </c>
       <c r="H19" s="23" t="inlineStr">
@@ -38205,7 +38205,7 @@
       </c>
       <c r="G24" s="23" t="inlineStr">
         <is>
-          <t>30-Dec-2024 (Mon)</t>
+          <t>31-Dec-2024 (Tue)</t>
         </is>
       </c>
       <c r="H24" s="23" t="inlineStr">
@@ -38367,7 +38367,7 @@
       </c>
       <c r="G26" s="23" t="inlineStr">
         <is>
-          <t>19-Nov-2024 (Tue)</t>
+          <t>20-Nov-2024 (Wed)</t>
         </is>
       </c>
       <c r="H26" s="23" t="inlineStr">
@@ -38691,7 +38691,7 @@
       </c>
       <c r="G30" s="23" t="inlineStr">
         <is>
-          <t>18-Nov-2024 (Mon)</t>
+          <t>19-Nov-2024 (Tue)</t>
         </is>
       </c>
       <c r="H30" s="23" t="inlineStr">
@@ -39091,7 +39091,7 @@
       </c>
       <c r="F35" s="23" t="inlineStr">
         <is>
-          <t>13-Nov-2024 (Wed)</t>
+          <t>12-Nov-2024 (Tue)</t>
         </is>
       </c>
       <c r="G35" s="23" t="inlineStr">
@@ -39501,7 +39501,7 @@
       </c>
       <c r="G40" s="23" t="inlineStr">
         <is>
-          <t>20-Nov-2024 (Wed)</t>
+          <t>21-Nov-2024 (Thu)</t>
         </is>
       </c>
       <c r="H40" s="23" t="inlineStr">
@@ -39820,7 +39820,7 @@
       </c>
       <c r="F44" s="23" t="inlineStr">
         <is>
-          <t>11-Nov-2024 (Mon)</t>
+          <t>08-Nov-2024 (Fri)</t>
         </is>
       </c>
       <c r="G44" s="23" t="inlineStr">
@@ -40063,7 +40063,7 @@
       </c>
       <c r="F47" s="23" t="inlineStr">
         <is>
-          <t>11-Nov-2024 (Mon)</t>
+          <t>08-Nov-2024 (Fri)</t>
         </is>
       </c>
       <c r="G47" s="23" t="inlineStr">
@@ -40144,7 +40144,7 @@
       </c>
       <c r="F48" s="23" t="inlineStr">
         <is>
-          <t>11-Nov-2024 (Mon)</t>
+          <t>08-Nov-2024 (Fri)</t>
         </is>
       </c>
       <c r="G48" s="23" t="inlineStr">
@@ -40230,7 +40230,7 @@
       </c>
       <c r="G49" s="23" t="inlineStr">
         <is>
-          <t>25-Dec-2024 (Wed)</t>
+          <t>26-Dec-2024 (Thu)</t>
         </is>
       </c>
       <c r="H49" s="23" t="inlineStr">
@@ -40387,12 +40387,12 @@
       </c>
       <c r="F51" s="23" t="inlineStr">
         <is>
-          <t>31-Oct-2024 (Thu)</t>
+          <t>30-Oct-2024 (Wed)</t>
         </is>
       </c>
       <c r="G51" s="23" t="inlineStr">
         <is>
-          <t>18-Nov-2024 (Mon)</t>
+          <t>19-Nov-2024 (Tue)</t>
         </is>
       </c>
       <c r="H51" s="23" t="inlineStr">
@@ -40468,7 +40468,7 @@
       </c>
       <c r="F52" s="23" t="inlineStr">
         <is>
-          <t>11-Nov-2024 (Mon)</t>
+          <t>08-Nov-2024 (Fri)</t>
         </is>
       </c>
       <c r="G52" s="23" t="inlineStr">
@@ -40635,7 +40635,7 @@
       </c>
       <c r="G54" s="23" t="inlineStr">
         <is>
-          <t>25-Dec-2024 (Wed)</t>
+          <t>26-Dec-2024 (Thu)</t>
         </is>
       </c>
       <c r="H54" s="23" t="inlineStr">
@@ -40711,7 +40711,7 @@
       </c>
       <c r="F55" s="23" t="inlineStr">
         <is>
-          <t>13-Nov-2024 (Wed)</t>
+          <t>12-Nov-2024 (Tue)</t>
         </is>
       </c>
       <c r="G55" s="23" t="inlineStr">
@@ -41176,7 +41176,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -41532,7 +41532,7 @@
       </c>
       <c r="G11" s="23" t="inlineStr">
         <is>
-          <t>19-Mar-2025 (Wed)</t>
+          <t>20-Mar-2025 (Thu)</t>
         </is>
       </c>
       <c r="H11" s="23" t="inlineStr">
@@ -41613,7 +41613,7 @@
       </c>
       <c r="G12" s="23" t="inlineStr">
         <is>
-          <t>27-Feb-2025 (Thu)</t>
+          <t>28-Feb-2025 (Fri)</t>
         </is>
       </c>
       <c r="H12" s="23" t="inlineStr">
@@ -41775,7 +41775,7 @@
       </c>
       <c r="G14" s="23" t="inlineStr">
         <is>
-          <t>19-Mar-2025 (Wed)</t>
+          <t>20-Mar-2025 (Thu)</t>
         </is>
       </c>
       <c r="H14" s="23" t="inlineStr">
@@ -41856,7 +41856,7 @@
       </c>
       <c r="G15" s="23" t="inlineStr">
         <is>
-          <t>28-Feb-2025 (Fri)</t>
+          <t>03-Mar-2025 (Mon)</t>
         </is>
       </c>
       <c r="H15" s="23" t="inlineStr">
@@ -42094,7 +42094,7 @@
       </c>
       <c r="F18" s="23" t="inlineStr">
         <is>
-          <t>11-Mar-2025 (Tue)</t>
+          <t>10-Mar-2025 (Mon)</t>
         </is>
       </c>
       <c r="G18" s="23" t="inlineStr">
@@ -42342,7 +42342,7 @@
       </c>
       <c r="G21" s="23" t="inlineStr">
         <is>
-          <t>14-Mar-2025 (Fri)</t>
+          <t>17-Mar-2025 (Mon)</t>
         </is>
       </c>
       <c r="H21" s="23" t="inlineStr">
@@ -42823,7 +42823,7 @@
       </c>
       <c r="F27" s="23" t="inlineStr">
         <is>
-          <t>10-Mar-2025 (Mon)</t>
+          <t>07-Mar-2025 (Fri)</t>
         </is>
       </c>
       <c r="G27" s="23" t="inlineStr">
@@ -42904,7 +42904,7 @@
       </c>
       <c r="F28" s="23" t="inlineStr">
         <is>
-          <t>14-Mar-2025 (Fri)</t>
+          <t>13-Mar-2025 (Thu)</t>
         </is>
       </c>
       <c r="G28" s="23" t="inlineStr">
@@ -43071,7 +43071,7 @@
       </c>
       <c r="G30" s="23" t="inlineStr">
         <is>
-          <t>27-Feb-2025 (Thu)</t>
+          <t>28-Feb-2025 (Fri)</t>
         </is>
       </c>
       <c r="H30" s="23" t="inlineStr">
@@ -43152,7 +43152,7 @@
       </c>
       <c r="G31" s="23" t="inlineStr">
         <is>
-          <t>14-Mar-2025 (Fri)</t>
+          <t>17-Mar-2025 (Mon)</t>
         </is>
       </c>
       <c r="H31" s="23" t="inlineStr">
@@ -43390,7 +43390,7 @@
       </c>
       <c r="F34" s="23" t="inlineStr">
         <is>
-          <t>14-Mar-2025 (Fri)</t>
+          <t>13-Mar-2025 (Thu)</t>
         </is>
       </c>
       <c r="G34" s="23" t="inlineStr">
@@ -43471,7 +43471,7 @@
       </c>
       <c r="F35" s="23" t="inlineStr">
         <is>
-          <t>11-Mar-2025 (Tue)</t>
+          <t>10-Mar-2025 (Mon)</t>
         </is>
       </c>
       <c r="G35" s="23" t="inlineStr">
@@ -43638,7 +43638,7 @@
       </c>
       <c r="G37" s="23" t="inlineStr">
         <is>
-          <t>14-Mar-2025 (Fri)</t>
+          <t>17-Mar-2025 (Mon)</t>
         </is>
       </c>
       <c r="H37" s="23" t="inlineStr">
@@ -43714,7 +43714,7 @@
       </c>
       <c r="F38" s="23" t="inlineStr">
         <is>
-          <t>12-Mar-2025 (Wed)</t>
+          <t>11-Mar-2025 (Tue)</t>
         </is>
       </c>
       <c r="G38" s="23" t="inlineStr">
@@ -44524,7 +44524,7 @@
       </c>
       <c r="F48" s="23" t="inlineStr">
         <is>
-          <t>14-Mar-2025 (Fri)</t>
+          <t>13-Mar-2025 (Thu)</t>
         </is>
       </c>
       <c r="G48" s="23" t="inlineStr">
@@ -45010,7 +45010,7 @@
       </c>
       <c r="F54" s="23" t="inlineStr">
         <is>
-          <t>07-Mar-2025 (Fri)</t>
+          <t>06-Mar-2025 (Thu)</t>
         </is>
       </c>
       <c r="G54" s="23" t="inlineStr">
@@ -45253,7 +45253,7 @@
       </c>
       <c r="F57" s="23" t="inlineStr">
         <is>
-          <t>07-Mar-2025 (Fri)</t>
+          <t>06-Mar-2025 (Thu)</t>
         </is>
       </c>
       <c r="G57" s="23" t="inlineStr">
@@ -45415,7 +45415,7 @@
       </c>
       <c r="F59" s="23" t="inlineStr">
         <is>
-          <t>10-Mar-2025 (Mon)</t>
+          <t>07-Mar-2025 (Fri)</t>
         </is>
       </c>
       <c r="G59" s="23" t="inlineStr">
@@ -45556,7 +45556,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -45826,12 +45826,12 @@
       </c>
       <c r="F10" s="23" t="inlineStr">
         <is>
-          <t>08-Apr-2025 (Tue)</t>
+          <t>07-Apr-2025 (Mon)</t>
         </is>
       </c>
       <c r="G10" s="23" t="inlineStr">
         <is>
-          <t>16-Apr-2025 (Wed)</t>
+          <t>17-Apr-2025 (Thu)</t>
         </is>
       </c>
       <c r="H10" s="23" t="inlineStr">
@@ -45993,7 +45993,7 @@
       </c>
       <c r="G12" s="23" t="inlineStr">
         <is>
-          <t>16-Apr-2025 (Wed)</t>
+          <t>17-Apr-2025 (Thu)</t>
         </is>
       </c>
       <c r="H12" s="23" t="inlineStr">
@@ -46069,7 +46069,7 @@
       </c>
       <c r="F13" s="23" t="inlineStr">
         <is>
-          <t>17-Apr-2025 (Thu)</t>
+          <t>16-Apr-2025 (Wed)</t>
         </is>
       </c>
       <c r="G13" s="23" t="inlineStr">
@@ -46555,7 +46555,7 @@
       </c>
       <c r="F19" s="23" t="inlineStr">
         <is>
-          <t>16-Apr-2025 (Wed)</t>
+          <t>15-Apr-2025 (Tue)</t>
         </is>
       </c>
       <c r="G19" s="23" t="inlineStr">
@@ -46636,7 +46636,7 @@
       </c>
       <c r="F20" s="23" t="inlineStr">
         <is>
-          <t>14-Apr-2025 (Mon)</t>
+          <t>09-Apr-2025 (Wed)</t>
         </is>
       </c>
       <c r="G20" s="23" t="inlineStr">
@@ -46960,12 +46960,12 @@
       </c>
       <c r="F24" s="23" t="inlineStr">
         <is>
-          <t>08-Apr-2025 (Tue)</t>
+          <t>07-Apr-2025 (Mon)</t>
         </is>
       </c>
       <c r="G24" s="23" t="inlineStr">
         <is>
-          <t>14-Apr-2025 (Mon)</t>
+          <t>15-Apr-2025 (Tue)</t>
         </is>
       </c>
       <c r="H24" s="23" t="inlineStr">
@@ -47122,12 +47122,12 @@
       </c>
       <c r="F26" s="23" t="inlineStr">
         <is>
-          <t>04-Apr-2025 (Fri)</t>
+          <t>03-Apr-2025 (Thu)</t>
         </is>
       </c>
       <c r="G26" s="23" t="inlineStr">
         <is>
-          <t>15-Apr-2025 (Tue)</t>
+          <t>16-Apr-2025 (Wed)</t>
         </is>
       </c>
       <c r="H26" s="23" t="inlineStr">
@@ -47203,7 +47203,7 @@
       </c>
       <c r="F27" s="23" t="inlineStr">
         <is>
-          <t>15-Apr-2025 (Tue)</t>
+          <t>11-Apr-2025 (Fri)</t>
         </is>
       </c>
       <c r="G27" s="23" t="inlineStr">
@@ -47365,7 +47365,7 @@
       </c>
       <c r="F29" s="23" t="inlineStr">
         <is>
-          <t>16-Apr-2025 (Wed)</t>
+          <t>15-Apr-2025 (Tue)</t>
         </is>
       </c>
       <c r="G29" s="23" t="inlineStr">
@@ -47851,12 +47851,12 @@
       </c>
       <c r="F35" s="23" t="inlineStr">
         <is>
-          <t>08-Apr-2025 (Tue)</t>
+          <t>07-Apr-2025 (Mon)</t>
         </is>
       </c>
       <c r="G35" s="23" t="inlineStr">
         <is>
-          <t>14-Apr-2025 (Mon)</t>
+          <t>15-Apr-2025 (Tue)</t>
         </is>
       </c>
       <c r="H35" s="23" t="inlineStr">
@@ -47937,7 +47937,7 @@
       </c>
       <c r="G36" s="23" t="inlineStr">
         <is>
-          <t>17-Apr-2025 (Thu)</t>
+          <t>21-Apr-2025 (Mon)</t>
         </is>
       </c>
       <c r="H36" s="23" t="inlineStr">
@@ -48499,12 +48499,12 @@
       </c>
       <c r="F43" s="23" t="inlineStr">
         <is>
-          <t>11-Apr-2025 (Fri)</t>
+          <t>09-Apr-2025 (Wed)</t>
         </is>
       </c>
       <c r="G43" s="23" t="inlineStr">
         <is>
-          <t>21-Apr-2025 (Mon)</t>
+          <t>22-Apr-2025 (Tue)</t>
         </is>
       </c>
       <c r="H43" s="23" t="inlineStr">
@@ -48742,12 +48742,12 @@
       </c>
       <c r="F46" s="23" t="inlineStr">
         <is>
-          <t>09-Apr-2025 (Wed)</t>
+          <t>07-Apr-2025 (Mon)</t>
         </is>
       </c>
       <c r="G46" s="23" t="inlineStr">
         <is>
-          <t>21-Apr-2025 (Mon)</t>
+          <t>22-Apr-2025 (Tue)</t>
         </is>
       </c>
       <c r="H46" s="23" t="inlineStr">
@@ -48985,12 +48985,12 @@
       </c>
       <c r="F49" s="23" t="inlineStr">
         <is>
-          <t>04-Apr-2025 (Fri)</t>
+          <t>03-Apr-2025 (Thu)</t>
         </is>
       </c>
       <c r="G49" s="23" t="inlineStr">
         <is>
-          <t>15-Apr-2025 (Tue)</t>
+          <t>16-Apr-2025 (Wed)</t>
         </is>
       </c>
       <c r="H49" s="23" t="inlineStr">
@@ -49633,7 +49633,7 @@
       </c>
       <c r="F57" s="23" t="inlineStr">
         <is>
-          <t>16-Apr-2025 (Wed)</t>
+          <t>15-Apr-2025 (Tue)</t>
         </is>
       </c>
       <c r="G57" s="23" t="inlineStr">
@@ -49795,12 +49795,12 @@
       </c>
       <c r="F59" s="23" t="inlineStr">
         <is>
-          <t>09-Apr-2025 (Wed)</t>
+          <t>07-Apr-2025 (Mon)</t>
         </is>
       </c>
       <c r="G59" s="23" t="inlineStr">
         <is>
-          <t>21-Apr-2025 (Mon)</t>
+          <t>22-Apr-2025 (Tue)</t>
         </is>
       </c>
       <c r="H59" s="23" t="inlineStr">
@@ -49936,7 +49936,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -50535,7 +50535,7 @@
       </c>
       <c r="G14" s="23" t="inlineStr">
         <is>
-          <t>18-Aug-2025 (Mon)</t>
+          <t>19-Aug-2025 (Tue)</t>
         </is>
       </c>
       <c r="H14" s="23" t="inlineStr">
@@ -50778,7 +50778,7 @@
       </c>
       <c r="G17" s="23" t="inlineStr">
         <is>
-          <t>27-Aug-2025 (Wed)</t>
+          <t>28-Aug-2025 (Thu)</t>
         </is>
       </c>
       <c r="H17" s="23" t="inlineStr">
@@ -50854,7 +50854,7 @@
       </c>
       <c r="F18" s="23" t="inlineStr">
         <is>
-          <t>12-Aug-2025 (Tue)</t>
+          <t>11-Aug-2025 (Mon)</t>
         </is>
       </c>
       <c r="G18" s="23" t="inlineStr">
@@ -51259,7 +51259,7 @@
       </c>
       <c r="F23" s="23" t="inlineStr">
         <is>
-          <t>11-Aug-2025 (Mon)</t>
+          <t>08-Aug-2025 (Fri)</t>
         </is>
       </c>
       <c r="G23" s="23" t="inlineStr">
@@ -51750,7 +51750,7 @@
       </c>
       <c r="G29" s="23" t="inlineStr">
         <is>
-          <t>18-Aug-2025 (Mon)</t>
+          <t>19-Aug-2025 (Tue)</t>
         </is>
       </c>
       <c r="H29" s="23" t="inlineStr">
@@ -52150,7 +52150,7 @@
       </c>
       <c r="F34" s="23" t="inlineStr">
         <is>
-          <t>07-Aug-2025 (Thu)</t>
+          <t>06-Aug-2025 (Wed)</t>
         </is>
       </c>
       <c r="G34" s="23" t="inlineStr">
@@ -52312,7 +52312,7 @@
       </c>
       <c r="F36" s="23" t="inlineStr">
         <is>
-          <t>14-Aug-2025 (Thu)</t>
+          <t>13-Aug-2025 (Wed)</t>
         </is>
       </c>
       <c r="G36" s="23" t="inlineStr">
@@ -52479,7 +52479,7 @@
       </c>
       <c r="G38" s="23" t="inlineStr">
         <is>
-          <t>21-Aug-2025 (Thu)</t>
+          <t>22-Aug-2025 (Fri)</t>
         </is>
       </c>
       <c r="H38" s="23" t="inlineStr">
@@ -52555,7 +52555,7 @@
       </c>
       <c r="F39" s="23" t="inlineStr">
         <is>
-          <t>14-Aug-2025 (Thu)</t>
+          <t>13-Aug-2025 (Wed)</t>
         </is>
       </c>
       <c r="G39" s="23" t="inlineStr">
@@ -52803,7 +52803,7 @@
       </c>
       <c r="G42" s="23" t="inlineStr">
         <is>
-          <t>29-Aug-2025 (Fri)</t>
+          <t>01-Sep-2025 (Mon)</t>
         </is>
       </c>
       <c r="H42" s="23" t="inlineStr">
@@ -52879,7 +52879,7 @@
       </c>
       <c r="F43" s="23" t="inlineStr">
         <is>
-          <t>14-Aug-2025 (Thu)</t>
+          <t>13-Aug-2025 (Wed)</t>
         </is>
       </c>
       <c r="G43" s="23" t="inlineStr">
@@ -53613,7 +53613,7 @@
       </c>
       <c r="G52" s="23" t="inlineStr">
         <is>
-          <t>18-Aug-2025 (Mon)</t>
+          <t>19-Aug-2025 (Tue)</t>
         </is>
       </c>
       <c r="H52" s="23" t="inlineStr">
@@ -54175,7 +54175,7 @@
       </c>
       <c r="F59" s="23" t="inlineStr">
         <is>
-          <t>14-Aug-2025 (Thu)</t>
+          <t>13-Aug-2025 (Wed)</t>
         </is>
       </c>
       <c r="G59" s="23" t="inlineStr">

</xml_diff>